<commit_message>
Updated README.md, task-board.xlsx and tasks.md
</commit_message>
<xml_diff>
--- a/docs/sprint2/task-board.xlsx
+++ b/docs/sprint2/task-board.xlsx
@@ -303,9 +303,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -355,7 +355,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -559,11 +559,11 @@
       <c r="F2" s="2">
         <v>2</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>14</v>
+      <c r="G2" s="2" t="str">
+        <v>Готово</v>
+      </c>
+      <c r="H2" s="2" t="str">
+        <v>requirements-defects.xlsx / Розподіл розділів; audit_questions.md</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>15</v>
@@ -588,8 +588,8 @@
       <c r="F3" s="2">
         <v>2.5</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>20</v>
+      <c r="G3" s="2" t="str">
+        <v>Готово</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>60</v>
@@ -602,8 +602,8 @@
       <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>23</v>
+      <c r="B4" s="2" t="str">
+        <v>Провести власну перевірку розділів 2, 3 і 5</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>24</v>
@@ -617,8 +617,8 @@
       <c r="F4" s="2">
         <v>2.5</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>20</v>
+      <c r="G4" s="2" t="str">
+        <v>Готово</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>61</v>
@@ -646,8 +646,8 @@
       <c r="F5" s="2">
         <v>2</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>20</v>
+      <c r="G5" s="2" t="str">
+        <v>Готово</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>62</v>
@@ -675,8 +675,8 @@
       <c r="F6" s="2">
         <v>3</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>20</v>
+      <c r="G6" s="2" t="str">
+        <v>Готово</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>63</v>
@@ -704,8 +704,8 @@
       <c r="F7" s="2">
         <v>4</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>13</v>
+      <c r="G7" s="2" t="str">
+        <v>Готово</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>32</v>
@@ -733,8 +733,8 @@
       <c r="F8" s="2">
         <v>2.5</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>20</v>
+      <c r="G8" s="2" t="str">
+        <v>Готово</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>35</v>
@@ -762,8 +762,8 @@
       <c r="F9" s="2">
         <v>5</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>13</v>
+      <c r="G9" s="2" t="str">
+        <v>Готово</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>38</v>
@@ -791,8 +791,8 @@
       <c r="F10" s="2">
         <v>6</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>13</v>
+      <c r="G10" s="2" t="str">
+        <v>Готово</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>41</v>
@@ -820,8 +820,8 @@
       <c r="F11" s="2">
         <v>2</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>20</v>
+      <c r="G11" s="2" t="str">
+        <v>Готово</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>44</v>
@@ -831,11 +831,6 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="G2:G11">
-      <formula1>"заплановано,в роботі,на рецензії,готово,перенесено,до виконання після Demo"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -890,7 +885,7 @@
       </c>
       <c r="B5" s="2">
         <f>COUNTIF(Задачі!G2:G11,"на рецензії")</f>
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="36" customHeight="1">

</xml_diff>